<commit_message>
Algorithm works, and gives somewhat logical graph, but physically, dosent make that much sense because pressures are going over the bigger Psat, which dosent make sense
</commit_message>
<xml_diff>
--- a/Asignacion 2/Asignacion 2.xlsx
+++ b/Asignacion 2/Asignacion 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30021"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30103"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5f906da8c23dd95/Desktop/Icesi_Pregrado/2026-1/termo 2/Asignacion 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2419" documentId="11_F25DC773A252ABDACC10485489D862385BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EBB07BE-C23A-4658-B128-772DDEB69FB8}"/>
+  <xr:revisionPtr revIDLastSave="2422" documentId="11_F25DC773A252ABDACC10485489D862385BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99BDC34F-C835-487F-BFED-E10666F04DB1}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="12" yWindow="12" windowWidth="23016" windowHeight="12216" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Punto 2" sheetId="1" r:id="rId1"/>
@@ -289,27 +289,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -326,15 +314,26 @@
     <xf numFmtId="2" fontId="2" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -628,6 +627,80 @@
     </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>313052</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>129710</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CFBB8519-919E-F7B5-BA6E-53AA035FED1F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6248400" y="4206240"/>
+          <a:ext cx="7292972" cy="1958510"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF">
+            <a:shade val="85000"/>
+          </a:srgbClr>
+        </a:solidFill>
+        <a:ln w="88900" cap="sq">
+          <a:solidFill>
+            <a:srgbClr val="FFFFFF"/>
+          </a:solidFill>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:effectLst>
+          <a:outerShdw blurRad="55000" dist="18000" dir="5400000" algn="tl" rotWithShape="0">
+            <a:srgbClr val="000000">
+              <a:alpha val="40000"/>
+            </a:srgbClr>
+          </a:outerShdw>
+        </a:effectLst>
+        <a:scene3d>
+          <a:camera prst="orthographicFront"/>
+          <a:lightRig rig="twoPt" dir="t">
+            <a:rot lat="0" lon="0" rev="7200000"/>
+          </a:lightRig>
+        </a:scene3d>
+        <a:sp3d>
+          <a:bevelT w="25400" h="19050"/>
+          <a:contourClr>
+            <a:srgbClr val="FFFFFF"/>
+          </a:contourClr>
+        </a:sp3d>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -909,15 +982,15 @@
       <c r="B1" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="6" t="s">
+      <c r="D1" s="27"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="6"/>
+      <c r="G1" s="26"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
@@ -933,7 +1006,7 @@
       <c r="E2" s="1">
         <v>3</v>
       </c>
-      <c r="F2" s="15">
+      <c r="F2" s="11">
         <v>4</v>
       </c>
       <c r="G2" s="3">
@@ -943,7 +1016,7 @@
       <c r="M2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="10" t="s">
         <v>17</v>
       </c>
       <c r="O2" s="3" t="s">
@@ -954,35 +1027,35 @@
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="24">
+      <c r="B3" s="20">
         <v>1.0233000000000001</v>
       </c>
       <c r="C3" s="2">
         <v>0.45</v>
       </c>
-      <c r="D3" s="19">
+      <c r="D3" s="15">
         <f>(B3*C3/(1-B$9))/(B$11+(B3*B$9/(1-B$9)))</f>
         <v>0.42575730093353503</v>
       </c>
-      <c r="E3" s="19">
+      <c r="E3" s="15">
         <f>(C3-D3*B$9)/(1-B$9)</f>
         <v>0.45891752460636082</v>
       </c>
-      <c r="F3" s="20">
+      <c r="F3" s="16">
         <f>(B3*E3/(1-B$15))/(B$17+(B3*B$15/(1-B$15)))</f>
         <v>0.48640784641347651</v>
       </c>
-      <c r="G3" s="19">
+      <c r="G3" s="15">
         <f>E3/(B$15*((B3/B$17)-1)+1)</f>
         <v>0.44713595811759699</v>
       </c>
       <c r="M3" s="2">
         <v>0.39430681820000002</v>
       </c>
-      <c r="N3" s="10">
+      <c r="N3" s="7">
         <v>1.0233000000000001</v>
       </c>
-      <c r="O3" s="9">
+      <c r="O3" s="6">
         <v>1022</v>
       </c>
     </row>
@@ -990,35 +1063,35 @@
       <c r="A4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="23">
+      <c r="B4" s="19">
         <v>2.7599</v>
       </c>
       <c r="C4" s="2">
         <v>0.25</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="22">
         <f t="shared" ref="D4:D5" si="0">(B4*C4/(1-B$9))/(B$11+(B4*B$9/(1-B$9)))</f>
         <v>0.44555409134576213</v>
       </c>
-      <c r="E4" s="19">
+      <c r="E4" s="15">
         <f t="shared" ref="E4:E5" si="1">(C4-D4*B$9)/(1-B$9)</f>
         <v>0.17806665558693263</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="22">
         <f>(B4*E4/(1-B$15))/(B$17+(B4*B$15/(1-B$15)))</f>
         <v>0.3306182118393115</v>
       </c>
-      <c r="G4" s="19">
+      <c r="G4" s="15">
         <f t="shared" ref="G4:G5" si="2">E4/(B$15*((B4/B$17)-1)+1)</f>
         <v>0.112687417193056</v>
       </c>
       <c r="M4" s="2">
         <v>0.2753395522</v>
       </c>
-      <c r="N4" s="10">
+      <c r="N4" s="7">
         <v>2.7599</v>
       </c>
-      <c r="O4" s="9">
+      <c r="O4" s="6">
         <v>2758</v>
       </c>
     </row>
@@ -1026,32 +1099,32 @@
       <c r="A5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="25">
+      <c r="B5" s="21">
         <v>0.39101999999999998</v>
       </c>
       <c r="C5" s="2">
         <v>0.3</v>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="15">
         <f t="shared" si="0"/>
         <v>0.12869094287060745</v>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="15">
         <f t="shared" si="1"/>
         <v>0.36301496083647894</v>
       </c>
-      <c r="F5" s="20">
+      <c r="F5" s="16">
         <f>(B5*E5/(1-B$15))/(B$17+(B5*B$15/(1-B$15)))</f>
         <v>0.18297161509753049</v>
       </c>
-      <c r="G5" s="19">
-        <f t="shared" si="2"/>
+      <c r="G5" s="15">
+        <f>E5/(B$15*((B5/B$17)-1)+1)</f>
         <v>0.44017639472459968</v>
       </c>
       <c r="M5" s="2">
         <v>0.39430681820000002</v>
       </c>
-      <c r="N5" s="10">
+      <c r="N5" s="7">
         <v>0.39101999999999998</v>
       </c>
       <c r="O5" s="2" t="s">
@@ -1069,19 +1142,19 @@
         <f>SUM(C3:C5)</f>
         <v>1</v>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="15">
         <f t="shared" ref="D6:E6" si="3">SUM(D3:D5)</f>
         <v>1.0000023351499046</v>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="15">
         <f t="shared" si="3"/>
         <v>0.99999914102977239</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="17">
         <f t="shared" ref="F6" si="4">SUM(F3:F5)</f>
         <v>0.99999767335031842</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="18">
         <f t="shared" ref="G6" si="5">SUM(G3:G5)</f>
         <v>0.99999977003525264</v>
       </c>
@@ -1106,7 +1179,7 @@
       <c r="D9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="14">
         <f>C3/(B$9*((B3/B$11) - 1) + 1)</f>
         <v>0.45891752460636087</v>
       </c>
@@ -1129,7 +1202,7 @@
       <c r="C10" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="14">
         <f>(C4/(B$9*(B4/B$11 - 1) + 1))</f>
         <v>0.17806665558693269</v>
       </c>
@@ -1144,44 +1217,44 @@
       <c r="C11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="14">
         <f>(C5/(B$9*(B5/B$11 - 1) + 1))</f>
         <v>0.36301496083647888</v>
       </c>
-      <c r="K11" s="12" t="s">
+      <c r="K11" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="L11" s="11" t="s">
+      <c r="L11" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="M11" s="12" t="s">
+      <c r="M11" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="N11" s="11" t="s">
+      <c r="N11" s="29" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C12" s="1"/>
-      <c r="E12" s="18" t="s">
+      <c r="E12" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="L12" s="11"/>
-      <c r="N12" s="11"/>
+      <c r="L12" s="29"/>
+      <c r="N12" s="29"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="C13" s="1"/>
-      <c r="E13" s="18"/>
-      <c r="L13" s="11"/>
-      <c r="N13" s="11"/>
+      <c r="E13" s="14"/>
+      <c r="L13" s="29"/>
+      <c r="N13" s="29"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C14" s="1"/>
-      <c r="E14" s="18"/>
-      <c r="O14" s="13">
+      <c r="E14" s="14"/>
+      <c r="O14" s="9">
         <v>5</v>
       </c>
     </row>
@@ -1197,7 +1270,7 @@
       <c r="D15" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="14">
         <f>(E3/(B$15*((B3/B$17) - 1) + 1))</f>
         <v>0.44713595811759699</v>
       </c>
@@ -1217,7 +1290,7 @@
       <c r="C16" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="14">
         <f t="shared" ref="E16:E17" si="6">(E4/(B$15*((B4/B$17) - 1) + 1))</f>
         <v>0.112687417193056</v>
       </c>
@@ -1226,19 +1299,19 @@
       <c r="A17" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B17" s="17">
+      <c r="B17" s="13">
         <v>0.94068019115133239</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="14">
         <f t="shared" si="6"/>
         <v>0.44017639472459968</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="E18" s="18"/>
+      <c r="E18" s="14"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="K19">
@@ -1250,7 +1323,7 @@
       <c r="B20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="K20" s="18">
+      <c r="K20" s="14">
         <f>K19+D25</f>
         <v>1.0000006279739528</v>
       </c>
@@ -1266,10 +1339,10 @@
       <c r="D21" s="3">
         <v>2</v>
       </c>
-      <c r="E21" s="27">
+      <c r="E21" s="3">
         <v>3</v>
       </c>
-      <c r="F21" s="15">
+      <c r="F21" s="11">
         <v>4</v>
       </c>
       <c r="G21" s="3">
@@ -1280,25 +1353,25 @@
       <c r="A22" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B22" s="24">
+      <c r="B22" s="20">
         <v>1.0233000000000001</v>
       </c>
       <c r="C22" s="2">
         <v>0.45</v>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="15">
         <f>(B22*C22/(1-B$9))*B9/(B$11+(B22*B$9/(1-B$9)))</f>
         <v>0.11449564529095456</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="15">
         <f>C3*(1-B$9)/(B$9*((B$3/B$11)-1)+1)</f>
         <v>0.33550435470904544</v>
       </c>
-      <c r="F22" s="20">
+      <c r="F22" s="16">
         <f>(B22*E22/(1-B$15))*(B15)/(B$17+(B22*B$15/(1-B$15)))</f>
         <v>0.10668057453875755</v>
       </c>
-      <c r="G22" s="19">
+      <c r="G22" s="15">
         <f>E22*(1-B15)/(B$15*((B22/B$17)-1)+1)</f>
         <v>0.2288237801702879</v>
       </c>
@@ -1307,25 +1380,25 @@
       <c r="A23" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B23" s="23">
+      <c r="B23" s="19">
         <v>2.7599</v>
       </c>
       <c r="C23" s="2">
         <v>0.25</v>
       </c>
-      <c r="D23" s="26">
+      <c r="D23" s="22">
         <f>(B23*C23/(1-B$9))*B9/(B$11+(B23*B$9/(1-B$9)))</f>
         <v>0.11981944429091949</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="15">
         <f>C4*(1-B$9)/(B$9*((B4/B$11)-1)+1)</f>
         <v>0.13018055570908052</v>
       </c>
-      <c r="F23" s="26">
+      <c r="F23" s="22">
         <f>(B23*E23/(1-B$15))*B15/(B$17+(B23*B$15/(1-B$15)))</f>
         <v>7.2512277612422155E-2</v>
       </c>
-      <c r="G23" s="19">
+      <c r="G23" s="15">
         <f>E23*(1-B15)/(B$15*((B23/B$17)-1)+1)</f>
         <v>5.7668278096658365E-2</v>
       </c>
@@ -1334,25 +1407,25 @@
       <c r="A24" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B24" s="25">
+      <c r="B24" s="21">
         <v>0.39101999999999998</v>
       </c>
       <c r="C24" s="2">
         <v>0.3</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="15">
         <f>(B24*C24/(1-B$9))*B9/(B$11+(B24*B$9/(1-B$9)))</f>
         <v>3.4607868179274692E-2</v>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="15">
         <f>C5*(1-B$9)/(B$9*((B5/B$11)-1)+1)</f>
         <v>0.2653921318207253</v>
       </c>
-      <c r="F24" s="20">
+      <c r="F24" s="16">
         <f>(B24*E24/(1-B$15))*B15/(B$17+(B24*B$15/(1-B$15)))</f>
         <v>4.0129938624172953E-2</v>
       </c>
-      <c r="G24" s="19">
+      <c r="G24" s="15">
         <f>E24*(1-B15)/(B$15*((B24/B$17)-1)+1)</f>
         <v>0.22526219319655233</v>
       </c>
@@ -1368,63 +1441,63 @@
         <f>SUM(C22:C24)</f>
         <v>1</v>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="15">
         <f t="shared" ref="D25:G25" si="7">SUM(D22:D24)</f>
         <v>0.26892295776114872</v>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="15">
         <f>SUM(E22:E24)</f>
         <v>0.73107704223885128</v>
       </c>
-      <c r="F25" s="21">
+      <c r="F25" s="17">
         <f t="shared" si="7"/>
         <v>0.21932279077535266</v>
       </c>
-      <c r="G25" s="22">
+      <c r="G25" s="18">
         <f t="shared" si="7"/>
         <v>0.51175425146349851</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="D27" s="18"/>
+      <c r="D27" s="14"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="15">
+      <c r="D29" s="11">
         <v>2</v>
       </c>
-      <c r="E29" s="29">
+      <c r="E29" s="24">
         <f>D23/C23</f>
         <v>0.47927777716367798</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C30" s="30" t="s">
+      <c r="C30" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="15">
+      <c r="D30" s="11">
         <v>4</v>
       </c>
-      <c r="E30" s="29">
+      <c r="E30" s="24">
         <f>F23/C23</f>
         <v>0.29004911044968862</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C31" s="30"/>
-      <c r="D31" s="15">
+      <c r="C31" s="25"/>
+      <c r="D31" s="11">
         <v>5</v>
       </c>
-      <c r="E31" s="29">
+      <c r="E31" s="24">
         <f>G23/C23</f>
         <v>0.23067311238663346</v>
       </c>

</xml_diff>